<commit_message>
Exam Excel: advance modul 2 Completed
</commit_message>
<xml_diff>
--- a/Exam/Excel/advanced_assessment_project/Raw_Transactions_2024_finish.xlsx
+++ b/Exam/Excel/advanced_assessment_project/Raw_Transactions_2024_finish.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\Project\Data-Analyst\Exam\Excel\advanced_assessment_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DDCA227-7C3A-4975-B1E0-40A6CF023DB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59A8E13B-F97A-4E0D-B2F6-BDDED7910EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{56521A79-FDF7-45C8-BAA3-ABC64B3F8849}"/>
   </bookViews>
@@ -18,6 +18,7 @@
   <externalReferences>
     <externalReference r:id="rId2"/>
     <externalReference r:id="rId3"/>
+    <externalReference r:id="rId4"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,8 +37,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="241">
   <si>
     <t>Trx_ID</t>
   </si>
@@ -739,13 +762,35 @@
   </si>
   <si>
     <t>Weight_KG</t>
+  </si>
+  <si>
+    <t>Customer_Region</t>
+  </si>
+  <si>
+    <t>Membership_Tier</t>
+  </si>
+  <si>
+    <t>Courier_Name</t>
+  </si>
+  <si>
+    <t>Service_Type</t>
+  </si>
+  <si>
+    <t>SLA_Days</t>
+  </si>
+  <si>
+    <t>Base_Rate_Per_KG</t>
+  </si>
+  <si>
+    <t>Sales_Commission_Rate</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
+    <numFmt numFmtId="42" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.E+00"/>
     <numFmt numFmtId="165" formatCode="&quot;Rp&quot;#,##0"/>
   </numFmts>
@@ -1247,7 +1292,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1255,6 +1300,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1334,6 +1380,12 @@
           <cell r="C2">
             <v>81234567890</v>
           </cell>
+          <cell r="D2" t="str">
+            <v>Jawa Barat</v>
+          </cell>
+          <cell r="G2" t="str">
+            <v>VIP</v>
+          </cell>
         </row>
         <row r="3">
           <cell r="A3" t="str">
@@ -1345,6 +1397,12 @@
           <cell r="C3">
             <v>628189876543</v>
           </cell>
+          <cell r="D3" t="str">
+            <v>DKI Jakarta</v>
+          </cell>
+          <cell r="G3" t="str">
+            <v>Gold</v>
+          </cell>
         </row>
         <row r="4">
           <cell r="A4" t="str">
@@ -1356,6 +1414,12 @@
           <cell r="C4">
             <v>6285611223344</v>
           </cell>
+          <cell r="D4" t="str">
+            <v>Jawa Tengah</v>
+          </cell>
+          <cell r="G4" t="str">
+            <v>Platinum</v>
+          </cell>
         </row>
         <row r="5">
           <cell r="A5" t="str">
@@ -1367,6 +1431,12 @@
           <cell r="C5">
             <v>87855443322</v>
           </cell>
+          <cell r="D5" t="str">
+            <v>Jawa Timur</v>
+          </cell>
+          <cell r="G5" t="str">
+            <v>Silver</v>
+          </cell>
         </row>
         <row r="6">
           <cell r="A6" t="str">
@@ -1378,6 +1448,12 @@
           <cell r="C6" t="str">
             <v>8189876543</v>
           </cell>
+          <cell r="D6" t="str">
+            <v>DKI Jakarta</v>
+          </cell>
+          <cell r="G6" t="str">
+            <v>Gold</v>
+          </cell>
         </row>
         <row r="7">
           <cell r="A7" t="str">
@@ -1389,6 +1465,12 @@
           <cell r="C7">
             <v>81122334455</v>
           </cell>
+          <cell r="D7" t="str">
+            <v>Banten</v>
+          </cell>
+          <cell r="G7" t="str">
+            <v>Silver</v>
+          </cell>
         </row>
         <row r="8">
           <cell r="A8" t="str">
@@ -1400,6 +1482,12 @@
           <cell r="C8">
             <v>628170099887</v>
           </cell>
+          <cell r="D8" t="str">
+            <v>DI Yogyakarta</v>
+          </cell>
+          <cell r="G8" t="str">
+            <v>Platinum</v>
+          </cell>
         </row>
         <row r="9">
           <cell r="A9" t="str">
@@ -1411,6 +1499,12 @@
           <cell r="C9">
             <v>85211447788</v>
           </cell>
+          <cell r="D9" t="str">
+            <v>Sumatera Utara</v>
+          </cell>
+          <cell r="G9" t="str">
+            <v>Gold</v>
+          </cell>
         </row>
         <row r="10">
           <cell r="A10" t="str">
@@ -1422,6 +1516,12 @@
           <cell r="C10" t="str">
             <v>+62 819 3322 1100</v>
           </cell>
+          <cell r="D10" t="str">
+            <v>Sulawesi Selatan</v>
+          </cell>
+          <cell r="G10" t="str">
+            <v>Silver</v>
+          </cell>
         </row>
         <row r="11">
           <cell r="A11" t="str">
@@ -1432,6 +1532,12 @@
           </cell>
           <cell r="C11">
             <v>81377665544</v>
+          </cell>
+          <cell r="D11" t="str">
+            <v>Bali</v>
+          </cell>
+          <cell r="G11" t="str">
+            <v>VIP</v>
           </cell>
         </row>
       </sheetData>
@@ -1794,6 +1900,125 @@
           </cell>
           <cell r="G16" t="str">
             <v>0.4</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Master_SLA_Shipping"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="2">
+          <cell r="A2" t="str">
+            <v>JNT-EXP</v>
+          </cell>
+          <cell r="B2" t="str">
+            <v>J&amp;T Express</v>
+          </cell>
+          <cell r="C2" t="str">
+            <v>Express</v>
+          </cell>
+          <cell r="D2">
+            <v>2</v>
+          </cell>
+          <cell r="E2">
+            <v>15000</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="A3" t="str">
+            <v>JNT-REG</v>
+          </cell>
+          <cell r="B3" t="str">
+            <v>J&amp;T Express</v>
+          </cell>
+          <cell r="C3" t="str">
+            <v>Regular</v>
+          </cell>
+          <cell r="D3">
+            <v>4</v>
+          </cell>
+          <cell r="E3">
+            <v>10000</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="A4" t="str">
+            <v>JNE-YES</v>
+          </cell>
+          <cell r="B4" t="str">
+            <v>JNE</v>
+          </cell>
+          <cell r="C4" t="str">
+            <v>Overnight</v>
+          </cell>
+          <cell r="D4">
+            <v>1</v>
+          </cell>
+          <cell r="E4">
+            <v>25000</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="A5" t="str">
+            <v>JNE-REG</v>
+          </cell>
+          <cell r="B5" t="str">
+            <v>JNE</v>
+          </cell>
+          <cell r="C5" t="str">
+            <v>Regular</v>
+          </cell>
+          <cell r="D5">
+            <v>3</v>
+          </cell>
+          <cell r="E5">
+            <v>12000</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="A6" t="str">
+            <v>SISEPAT-BEST</v>
+          </cell>
+          <cell r="B6" t="str">
+            <v>SiCepat</v>
+          </cell>
+          <cell r="C6" t="str">
+            <v>Express</v>
+          </cell>
+          <cell r="D6">
+            <v>2</v>
+          </cell>
+          <cell r="E6">
+            <v>16000</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="A7" t="str">
+            <v>SISEPAT-GOKIL</v>
+          </cell>
+          <cell r="B7" t="str">
+            <v>SiCepat</v>
+          </cell>
+          <cell r="C7" t="str">
+            <v>Cargo</v>
+          </cell>
+          <cell r="D7">
+            <v>5</v>
+          </cell>
+          <cell r="E7">
+            <v>8000</v>
           </cell>
         </row>
       </sheetData>
@@ -2119,7 +2344,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6A4B63D-0D46-44D9-8B15-778A85DACDCF}">
-  <dimension ref="A1:W101"/>
+  <dimension ref="A1:AD101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
@@ -2144,9 +2369,15 @@
     <col min="20" max="20" width="20.85546875" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="22" max="23" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="22.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2216,8 +2447,29 @@
       <c r="W1" s="3" t="s">
         <v>233</v>
       </c>
+      <c r="X1" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="Y1" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="AB1" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="AC1" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="AD1" s="3" t="s">
+        <v>240</v>
+      </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -2298,8 +2550,36 @@
         <f>_xlfn.XLOOKUP(P2,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.8</v>
       </c>
+      <c r="X2" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M2,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y2" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M2,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z2" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G2,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA2" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G2,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB2" s="1">
+        <f>_xlfn.XLOOKUP(G2,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC2" s="7">
+        <f>_xlfn.XLOOKUP(G2,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD2" s="1" t="e" cm="1">
+        <f t="array" ref="AD2:AD101">INDEX(MATCH(S2,S2:S101,0),MATCH(Y2:Y101,0))</f>
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>20</v>
       </c>
@@ -2380,8 +2660,35 @@
         <f>_xlfn.XLOOKUP(P3,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.3</v>
       </c>
+      <c r="X3" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M3,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Barat</v>
+      </c>
+      <c r="Y3" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M3,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z3" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G3,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA3" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G3,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB3" s="1">
+        <f>_xlfn.XLOOKUP(G3,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC3" s="7">
+        <f>_xlfn.XLOOKUP(G3,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD3" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>28</v>
       </c>
@@ -2462,8 +2769,35 @@
         <f>_xlfn.XLOOKUP(P4,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.1</v>
       </c>
+      <c r="X4" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M4,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y4" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M4,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z4" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G4,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA4" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G4,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB4" s="1">
+        <f>_xlfn.XLOOKUP(G4,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC4" s="7">
+        <f>_xlfn.XLOOKUP(G4,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD4" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
@@ -2544,8 +2878,35 @@
         <f>_xlfn.XLOOKUP(P5,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.35</v>
       </c>
+      <c r="X5" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M5,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y5" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M5,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z5" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G5,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA5" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G5,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB5" s="1">
+        <f>_xlfn.XLOOKUP(G5,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC5" s="7">
+        <f>_xlfn.XLOOKUP(G5,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD5" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>40</v>
       </c>
@@ -2626,8 +2987,35 @@
         <f>_xlfn.XLOOKUP(P6,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.12</v>
       </c>
+      <c r="X6" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M6,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y6" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M6,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z6" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G6,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA6" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G6,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Overnight</v>
+      </c>
+      <c r="AB6" s="1">
+        <f>_xlfn.XLOOKUP(G6,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>1</v>
+      </c>
+      <c r="AC6" s="7">
+        <f>_xlfn.XLOOKUP(G6,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>25000</v>
+      </c>
+      <c r="AD6" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>44</v>
       </c>
@@ -2708,8 +3096,35 @@
         <f>_xlfn.XLOOKUP(P7,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.12</v>
       </c>
+      <c r="X7" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M7,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y7" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M7,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z7" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G7,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA7" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G7,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB7" s="1">
+        <f>_xlfn.XLOOKUP(G7,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC7" s="7">
+        <f>_xlfn.XLOOKUP(G7,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD7" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>49</v>
       </c>
@@ -2790,8 +3205,35 @@
         <f>_xlfn.XLOOKUP(P8,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>4.5</v>
       </c>
+      <c r="X8" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M8,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y8" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M8,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z8" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G8,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA8" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G8,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Overnight</v>
+      </c>
+      <c r="AB8" s="1">
+        <f>_xlfn.XLOOKUP(G8,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>1</v>
+      </c>
+      <c r="AC8" s="7">
+        <f>_xlfn.XLOOKUP(G8,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>25000</v>
+      </c>
+      <c r="AD8" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>51</v>
       </c>
@@ -2872,8 +3314,35 @@
         <f>_xlfn.XLOOKUP(P9,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.12</v>
       </c>
+      <c r="X9" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M9,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Banten</v>
+      </c>
+      <c r="Y9" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M9,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z9" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G9,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA9" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G9,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB9" s="1">
+        <f>_xlfn.XLOOKUP(G9,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC9" s="7">
+        <f>_xlfn.XLOOKUP(G9,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD9" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>55</v>
       </c>
@@ -2954,8 +3423,35 @@
         <f>_xlfn.XLOOKUP(P10,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.25</v>
       </c>
+      <c r="X10" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M10,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Banten</v>
+      </c>
+      <c r="Y10" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M10,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z10" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G10,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA10" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G10,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB10" s="1">
+        <f>_xlfn.XLOOKUP(G10,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC10" s="7">
+        <f>_xlfn.XLOOKUP(G10,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD10" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>58</v>
       </c>
@@ -3036,8 +3532,35 @@
         <f>_xlfn.XLOOKUP(P11,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.8</v>
       </c>
+      <c r="X11" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M11,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y11" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M11,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z11" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G11,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA11" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G11,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB11" s="1">
+        <f>_xlfn.XLOOKUP(G11,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC11" s="7">
+        <f>_xlfn.XLOOKUP(G11,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD11" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>60</v>
       </c>
@@ -3118,8 +3641,35 @@
         <f>_xlfn.XLOOKUP(P12,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>1.2</v>
       </c>
+      <c r="X12" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M12,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y12" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M12,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z12" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G12,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA12" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G12,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB12" s="1">
+        <f>_xlfn.XLOOKUP(G12,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC12" s="7">
+        <f>_xlfn.XLOOKUP(G12,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD12" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>63</v>
       </c>
@@ -3200,8 +3750,35 @@
         <f>_xlfn.XLOOKUP(P13,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.2</v>
       </c>
+      <c r="X13" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M13,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Barat</v>
+      </c>
+      <c r="Y13" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M13,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z13" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G13,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA13" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G13,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB13" s="1">
+        <f>_xlfn.XLOOKUP(G13,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC13" s="7">
+        <f>_xlfn.XLOOKUP(G13,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD13" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>66</v>
       </c>
@@ -3282,8 +3859,35 @@
         <f>_xlfn.XLOOKUP(P14,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.8</v>
       </c>
+      <c r="X14" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M14,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Barat</v>
+      </c>
+      <c r="Y14" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M14,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z14" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G14,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA14" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G14,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB14" s="1">
+        <f>_xlfn.XLOOKUP(G14,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC14" s="7">
+        <f>_xlfn.XLOOKUP(G14,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD14" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>68</v>
       </c>
@@ -3364,8 +3968,35 @@
         <f>_xlfn.XLOOKUP(P15,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>1.2</v>
       </c>
+      <c r="X15" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M15,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y15" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M15,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z15" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G15,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA15" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G15,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB15" s="1">
+        <f>_xlfn.XLOOKUP(G15,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC15" s="7">
+        <f>_xlfn.XLOOKUP(G15,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD15" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>71</v>
       </c>
@@ -3446,8 +4077,35 @@
         <f>_xlfn.XLOOKUP(P16,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.4</v>
       </c>
+      <c r="X16" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M16,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Banten</v>
+      </c>
+      <c r="Y16" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M16,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z16" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G16,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA16" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G16,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB16" s="1">
+        <f>_xlfn.XLOOKUP(G16,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC16" s="7">
+        <f>_xlfn.XLOOKUP(G16,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD16" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>74</v>
       </c>
@@ -3528,8 +4186,35 @@
         <f>_xlfn.XLOOKUP(P17,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.1</v>
       </c>
+      <c r="X17" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M17,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y17" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M17,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z17" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G17,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA17" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G17,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB17" s="1">
+        <f>_xlfn.XLOOKUP(G17,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC17" s="7">
+        <f>_xlfn.XLOOKUP(G17,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD17" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>76</v>
       </c>
@@ -3610,8 +4295,35 @@
         <f>_xlfn.XLOOKUP(P18,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.4</v>
       </c>
+      <c r="X18" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M18,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y18" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M18,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z18" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G18,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA18" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G18,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB18" s="1">
+        <f>_xlfn.XLOOKUP(G18,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC18" s="7">
+        <f>_xlfn.XLOOKUP(G18,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD18" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>77</v>
       </c>
@@ -3692,8 +4404,35 @@
         <f>_xlfn.XLOOKUP(P19,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.25</v>
       </c>
+      <c r="X19" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M19,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y19" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M19,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z19" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G19,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA19" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G19,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB19" s="1">
+        <f>_xlfn.XLOOKUP(G19,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC19" s="7">
+        <f>_xlfn.XLOOKUP(G19,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD19" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>79</v>
       </c>
@@ -3774,8 +4513,35 @@
         <f>_xlfn.XLOOKUP(P20,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.25</v>
       </c>
+      <c r="X20" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M20,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Barat</v>
+      </c>
+      <c r="Y20" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M20,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z20" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G20,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA20" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G20,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB20" s="1">
+        <f>_xlfn.XLOOKUP(G20,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC20" s="7">
+        <f>_xlfn.XLOOKUP(G20,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD20" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>81</v>
       </c>
@@ -3856,8 +4622,35 @@
         <f>_xlfn.XLOOKUP(P21,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>4.5</v>
       </c>
+      <c r="X21" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M21,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Bali</v>
+      </c>
+      <c r="Y21" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M21,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z21" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G21,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA21" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G21,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB21" s="1">
+        <f>_xlfn.XLOOKUP(G21,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC21" s="7">
+        <f>_xlfn.XLOOKUP(G21,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD21" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>83</v>
       </c>
@@ -3938,8 +4731,35 @@
         <f>_xlfn.XLOOKUP(P22,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.35</v>
       </c>
+      <c r="X22" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M22,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DI Yogyakarta</v>
+      </c>
+      <c r="Y22" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M22,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z22" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G22,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA22" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G22,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB22" s="1">
+        <f>_xlfn.XLOOKUP(G22,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC22" s="7">
+        <f>_xlfn.XLOOKUP(G22,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD22" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>86</v>
       </c>
@@ -4020,8 +4840,35 @@
         <f>_xlfn.XLOOKUP(P23,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.15</v>
       </c>
+      <c r="X23" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M23,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y23" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M23,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z23" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G23,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA23" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G23,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB23" s="1">
+        <f>_xlfn.XLOOKUP(G23,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC23" s="7">
+        <f>_xlfn.XLOOKUP(G23,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD23" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>88</v>
       </c>
@@ -4102,8 +4949,35 @@
         <f>_xlfn.XLOOKUP(P24,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.2</v>
       </c>
+      <c r="X24" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M24,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Barat</v>
+      </c>
+      <c r="Y24" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M24,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z24" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G24,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA24" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G24,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB24" s="1">
+        <f>_xlfn.XLOOKUP(G24,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC24" s="7">
+        <f>_xlfn.XLOOKUP(G24,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD24" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>89</v>
       </c>
@@ -4184,8 +5058,35 @@
         <f>_xlfn.XLOOKUP(P25,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.4</v>
       </c>
+      <c r="X25" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M25,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DI Yogyakarta</v>
+      </c>
+      <c r="Y25" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M25,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z25" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G25,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA25" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G25,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB25" s="1">
+        <f>_xlfn.XLOOKUP(G25,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC25" s="7">
+        <f>_xlfn.XLOOKUP(G25,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD25" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>92</v>
       </c>
@@ -4266,8 +5167,35 @@
         <f>_xlfn.XLOOKUP(P26,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>1.2</v>
       </c>
+      <c r="X26" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M26,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sumatera Utara</v>
+      </c>
+      <c r="Y26" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M26,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z26" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G26,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA26" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G26,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB26" s="1">
+        <f>_xlfn.XLOOKUP(G26,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC26" s="7">
+        <f>_xlfn.XLOOKUP(G26,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD26" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>95</v>
       </c>
@@ -4348,8 +5276,35 @@
         <f>_xlfn.XLOOKUP(P27,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.15</v>
       </c>
+      <c r="X27" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M27,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sumatera Utara</v>
+      </c>
+      <c r="Y27" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M27,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z27" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G27,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA27" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G27,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB27" s="1">
+        <f>_xlfn.XLOOKUP(G27,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC27" s="7">
+        <f>_xlfn.XLOOKUP(G27,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD27" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>97</v>
       </c>
@@ -4430,8 +5385,35 @@
         <f>_xlfn.XLOOKUP(P28,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.35</v>
       </c>
+      <c r="X28" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M28,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y28" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M28,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z28" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G28,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA28" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G28,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB28" s="1">
+        <f>_xlfn.XLOOKUP(G28,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC28" s="7">
+        <f>_xlfn.XLOOKUP(G28,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD28" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>98</v>
       </c>
@@ -4512,8 +5494,35 @@
         <f>_xlfn.XLOOKUP(P29,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.9</v>
       </c>
+      <c r="X29" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M29,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sulawesi Selatan</v>
+      </c>
+      <c r="Y29" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M29,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z29" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G29,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA29" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G29,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB29" s="1">
+        <f>_xlfn.XLOOKUP(G29,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC29" s="7">
+        <f>_xlfn.XLOOKUP(G29,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD29" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>101</v>
       </c>
@@ -4594,8 +5603,35 @@
         <f>_xlfn.XLOOKUP(P30,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.8</v>
       </c>
+      <c r="X30" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M30,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y30" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M30,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z30" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G30,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA30" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G30,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB30" s="1">
+        <f>_xlfn.XLOOKUP(G30,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC30" s="7">
+        <f>_xlfn.XLOOKUP(G30,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD30" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>102</v>
       </c>
@@ -4676,8 +5712,35 @@
         <f>_xlfn.XLOOKUP(P31,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.9</v>
       </c>
+      <c r="X31" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M31,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y31" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M31,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z31" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G31,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA31" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G31,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB31" s="1">
+        <f>_xlfn.XLOOKUP(G31,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC31" s="7">
+        <f>_xlfn.XLOOKUP(G31,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD31" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>103</v>
       </c>
@@ -4758,8 +5821,35 @@
         <f>_xlfn.XLOOKUP(P32,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.4</v>
       </c>
+      <c r="X32" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M32,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y32" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M32,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z32" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G32,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA32" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G32,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB32" s="1">
+        <f>_xlfn.XLOOKUP(G32,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC32" s="7">
+        <f>_xlfn.XLOOKUP(G32,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD32" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>105</v>
       </c>
@@ -4840,8 +5930,35 @@
         <f>_xlfn.XLOOKUP(P33,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.25</v>
       </c>
+      <c r="X33" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M33,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Banten</v>
+      </c>
+      <c r="Y33" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M33,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z33" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G33,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA33" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G33,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB33" s="1">
+        <f>_xlfn.XLOOKUP(G33,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC33" s="7">
+        <f>_xlfn.XLOOKUP(G33,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD33" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>106</v>
       </c>
@@ -4922,8 +6039,35 @@
         <f>_xlfn.XLOOKUP(P34,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.8</v>
       </c>
+      <c r="X34" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M34,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y34" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M34,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z34" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G34,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA34" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G34,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB34" s="1">
+        <f>_xlfn.XLOOKUP(G34,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC34" s="7">
+        <f>_xlfn.XLOOKUP(G34,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD34" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>108</v>
       </c>
@@ -5004,8 +6148,35 @@
         <f>_xlfn.XLOOKUP(P35,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.4</v>
       </c>
+      <c r="X35" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M35,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y35" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M35,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z35" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G35,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA35" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G35,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB35" s="1">
+        <f>_xlfn.XLOOKUP(G35,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC35" s="7">
+        <f>_xlfn.XLOOKUP(G35,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD35" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>110</v>
       </c>
@@ -5086,8 +6257,35 @@
         <f>_xlfn.XLOOKUP(P36,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.9</v>
       </c>
+      <c r="X36" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M36,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y36" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M36,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z36" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G36,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA36" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G36,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB36" s="1">
+        <f>_xlfn.XLOOKUP(G36,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC36" s="7">
+        <f>_xlfn.XLOOKUP(G36,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD36" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>112</v>
       </c>
@@ -5168,8 +6366,35 @@
         <f>_xlfn.XLOOKUP(P37,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.1</v>
       </c>
+      <c r="X37" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M37,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Tengah</v>
+      </c>
+      <c r="Y37" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M37,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z37" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G37,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA37" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G37,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Overnight</v>
+      </c>
+      <c r="AB37" s="1">
+        <f>_xlfn.XLOOKUP(G37,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>1</v>
+      </c>
+      <c r="AC37" s="7">
+        <f>_xlfn.XLOOKUP(G37,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>25000</v>
+      </c>
+      <c r="AD37" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>114</v>
       </c>
@@ -5250,8 +6475,35 @@
         <f>_xlfn.XLOOKUP(P38,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.35</v>
       </c>
+      <c r="X38" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M38,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y38" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M38,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z38" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G38,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA38" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G38,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB38" s="1">
+        <f>_xlfn.XLOOKUP(G38,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC38" s="7">
+        <f>_xlfn.XLOOKUP(G38,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD38" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>116</v>
       </c>
@@ -5332,8 +6584,35 @@
         <f>_xlfn.XLOOKUP(P39,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.35</v>
       </c>
+      <c r="X39" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M39,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y39" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M39,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z39" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G39,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA39" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G39,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB39" s="1">
+        <f>_xlfn.XLOOKUP(G39,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC39" s="7">
+        <f>_xlfn.XLOOKUP(G39,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD39" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>118</v>
       </c>
@@ -5414,8 +6693,35 @@
         <f>_xlfn.XLOOKUP(P40,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.3</v>
       </c>
+      <c r="X40" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M40,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Barat</v>
+      </c>
+      <c r="Y40" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M40,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z40" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G40,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA40" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G40,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Overnight</v>
+      </c>
+      <c r="AB40" s="1">
+        <f>_xlfn.XLOOKUP(G40,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>1</v>
+      </c>
+      <c r="AC40" s="7">
+        <f>_xlfn.XLOOKUP(G40,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>25000</v>
+      </c>
+      <c r="AD40" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>121</v>
       </c>
@@ -5496,8 +6802,35 @@
         <f>_xlfn.XLOOKUP(P41,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.15</v>
       </c>
+      <c r="X41" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M41,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Bali</v>
+      </c>
+      <c r="Y41" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M41,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z41" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G41,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA41" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G41,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB41" s="1">
+        <f>_xlfn.XLOOKUP(G41,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC41" s="7">
+        <f>_xlfn.XLOOKUP(G41,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD41" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>123</v>
       </c>
@@ -5578,8 +6911,35 @@
         <f>_xlfn.XLOOKUP(P42,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.9</v>
       </c>
+      <c r="X42" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M42,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y42" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M42,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z42" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G42,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA42" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G42,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB42" s="1">
+        <f>_xlfn.XLOOKUP(G42,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC42" s="7">
+        <f>_xlfn.XLOOKUP(G42,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD42" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>124</v>
       </c>
@@ -5660,8 +7020,35 @@
         <f>_xlfn.XLOOKUP(P43,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.8</v>
       </c>
+      <c r="X43" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M43,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DI Yogyakarta</v>
+      </c>
+      <c r="Y43" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M43,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z43" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G43,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA43" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G43,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB43" s="1">
+        <f>_xlfn.XLOOKUP(G43,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC43" s="7">
+        <f>_xlfn.XLOOKUP(G43,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD43" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>126</v>
       </c>
@@ -5742,8 +7129,35 @@
         <f>_xlfn.XLOOKUP(P44,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.4</v>
       </c>
+      <c r="X44" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M44,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Barat</v>
+      </c>
+      <c r="Y44" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M44,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z44" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G44,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA44" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G44,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB44" s="1">
+        <f>_xlfn.XLOOKUP(G44,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC44" s="7">
+        <f>_xlfn.XLOOKUP(G44,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD44" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>128</v>
       </c>
@@ -5824,8 +7238,35 @@
         <f>_xlfn.XLOOKUP(P45,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.15</v>
       </c>
+      <c r="X45" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M45,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y45" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M45,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z45" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G45,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA45" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G45,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB45" s="1">
+        <f>_xlfn.XLOOKUP(G45,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC45" s="7">
+        <f>_xlfn.XLOOKUP(G45,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD45" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>130</v>
       </c>
@@ -5906,8 +7347,35 @@
         <f>_xlfn.XLOOKUP(P46,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.25</v>
       </c>
+      <c r="X46" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M46,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y46" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M46,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z46" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G46,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA46" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G46,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB46" s="1">
+        <f>_xlfn.XLOOKUP(G46,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC46" s="7">
+        <f>_xlfn.XLOOKUP(G46,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD46" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>132</v>
       </c>
@@ -5988,8 +7456,35 @@
         <f>_xlfn.XLOOKUP(P47,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.25</v>
       </c>
+      <c r="X47" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M47,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Bali</v>
+      </c>
+      <c r="Y47" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M47,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z47" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G47,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA47" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G47,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB47" s="1">
+        <f>_xlfn.XLOOKUP(G47,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC47" s="7">
+        <f>_xlfn.XLOOKUP(G47,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD47" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>134</v>
       </c>
@@ -6070,8 +7565,35 @@
         <f>_xlfn.XLOOKUP(P48,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.1</v>
       </c>
+      <c r="X48" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M48,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Tengah</v>
+      </c>
+      <c r="Y48" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M48,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z48" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G48,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA48" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G48,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB48" s="1">
+        <f>_xlfn.XLOOKUP(G48,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC48" s="7">
+        <f>_xlfn.XLOOKUP(G48,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD48" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>137</v>
       </c>
@@ -6152,8 +7674,35 @@
         <f>_xlfn.XLOOKUP(P49,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.15</v>
       </c>
+      <c r="X49" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M49,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sulawesi Selatan</v>
+      </c>
+      <c r="Y49" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M49,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z49" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G49,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA49" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G49,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB49" s="1">
+        <f>_xlfn.XLOOKUP(G49,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC49" s="7">
+        <f>_xlfn.XLOOKUP(G49,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD49" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>138</v>
       </c>
@@ -6234,8 +7783,35 @@
         <f>_xlfn.XLOOKUP(P50,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.1</v>
       </c>
+      <c r="X50" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M50,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y50" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M50,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z50" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G50,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA50" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G50,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB50" s="1">
+        <f>_xlfn.XLOOKUP(G50,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC50" s="7">
+        <f>_xlfn.XLOOKUP(G50,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD50" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>140</v>
       </c>
@@ -6316,8 +7892,35 @@
         <f>_xlfn.XLOOKUP(P51,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.25</v>
       </c>
+      <c r="X51" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M51,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y51" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M51,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z51" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G51,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA51" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G51,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB51" s="1">
+        <f>_xlfn.XLOOKUP(G51,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC51" s="7">
+        <f>_xlfn.XLOOKUP(G51,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD51" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>142</v>
       </c>
@@ -6398,8 +8001,35 @@
         <f>_xlfn.XLOOKUP(P52,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.3</v>
       </c>
+      <c r="X52" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M52,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y52" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M52,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z52" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G52,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA52" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G52,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB52" s="1">
+        <f>_xlfn.XLOOKUP(G52,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC52" s="7">
+        <f>_xlfn.XLOOKUP(G52,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD52" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>144</v>
       </c>
@@ -6480,8 +8110,35 @@
         <f>_xlfn.XLOOKUP(P53,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.8</v>
       </c>
+      <c r="X53" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M53,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Bali</v>
+      </c>
+      <c r="Y53" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M53,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z53" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G53,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA53" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G53,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB53" s="1">
+        <f>_xlfn.XLOOKUP(G53,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC53" s="7">
+        <f>_xlfn.XLOOKUP(G53,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD53" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>146</v>
       </c>
@@ -6562,8 +8219,35 @@
         <f>_xlfn.XLOOKUP(P54,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.1</v>
       </c>
+      <c r="X54" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M54,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sulawesi Selatan</v>
+      </c>
+      <c r="Y54" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M54,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z54" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G54,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA54" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G54,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB54" s="1">
+        <f>_xlfn.XLOOKUP(G54,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC54" s="7">
+        <f>_xlfn.XLOOKUP(G54,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD54" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>148</v>
       </c>
@@ -6644,8 +8328,35 @@
         <f>_xlfn.XLOOKUP(P55,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.8</v>
       </c>
+      <c r="X55" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M55,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DI Yogyakarta</v>
+      </c>
+      <c r="Y55" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M55,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z55" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G55,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA55" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G55,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB55" s="1">
+        <f>_xlfn.XLOOKUP(G55,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC55" s="7">
+        <f>_xlfn.XLOOKUP(G55,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD55" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>150</v>
       </c>
@@ -6726,8 +8437,35 @@
         <f>_xlfn.XLOOKUP(P56,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>1.2</v>
       </c>
+      <c r="X56" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M56,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sumatera Utara</v>
+      </c>
+      <c r="Y56" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M56,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z56" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G56,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA56" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G56,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB56" s="1">
+        <f>_xlfn.XLOOKUP(G56,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC56" s="7">
+        <f>_xlfn.XLOOKUP(G56,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD56" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>152</v>
       </c>
@@ -6808,8 +8546,35 @@
         <f>_xlfn.XLOOKUP(P57,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.4</v>
       </c>
+      <c r="X57" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M57,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DI Yogyakarta</v>
+      </c>
+      <c r="Y57" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M57,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z57" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G57,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA57" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G57,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB57" s="1">
+        <f>_xlfn.XLOOKUP(G57,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC57" s="7">
+        <f>_xlfn.XLOOKUP(G57,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD57" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>154</v>
       </c>
@@ -6890,8 +8655,35 @@
         <f>_xlfn.XLOOKUP(P58,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.1</v>
       </c>
+      <c r="X58" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M58,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Barat</v>
+      </c>
+      <c r="Y58" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M58,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z58" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G58,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA58" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G58,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB58" s="1">
+        <f>_xlfn.XLOOKUP(G58,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC58" s="7">
+        <f>_xlfn.XLOOKUP(G58,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD58" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>156</v>
       </c>
@@ -6972,8 +8764,35 @@
         <f>_xlfn.XLOOKUP(P59,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>4.5</v>
       </c>
+      <c r="X59" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M59,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y59" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M59,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z59" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G59,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA59" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G59,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB59" s="1">
+        <f>_xlfn.XLOOKUP(G59,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC59" s="7">
+        <f>_xlfn.XLOOKUP(G59,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD59" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>158</v>
       </c>
@@ -7054,8 +8873,35 @@
         <f>_xlfn.XLOOKUP(P60,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.8</v>
       </c>
+      <c r="X60" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M60,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Bali</v>
+      </c>
+      <c r="Y60" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M60,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z60" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G60,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA60" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G60,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB60" s="1">
+        <f>_xlfn.XLOOKUP(G60,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC60" s="7">
+        <f>_xlfn.XLOOKUP(G60,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD60" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>160</v>
       </c>
@@ -7136,8 +8982,35 @@
         <f>_xlfn.XLOOKUP(P61,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.1</v>
       </c>
+      <c r="X61" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M61,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Bali</v>
+      </c>
+      <c r="Y61" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M61,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z61" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G61,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA61" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G61,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB61" s="1">
+        <f>_xlfn.XLOOKUP(G61,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC61" s="7">
+        <f>_xlfn.XLOOKUP(G61,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD61" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>162</v>
       </c>
@@ -7218,8 +9091,35 @@
         <f>_xlfn.XLOOKUP(P62,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.12</v>
       </c>
+      <c r="X62" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M62,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DI Yogyakarta</v>
+      </c>
+      <c r="Y62" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M62,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z62" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G62,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA62" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G62,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB62" s="1">
+        <f>_xlfn.XLOOKUP(G62,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC62" s="7">
+        <f>_xlfn.XLOOKUP(G62,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD62" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>163</v>
       </c>
@@ -7300,8 +9200,35 @@
         <f>_xlfn.XLOOKUP(P63,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>4.5</v>
       </c>
+      <c r="X63" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M63,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y63" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M63,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z63" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G63,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA63" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G63,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB63" s="1">
+        <f>_xlfn.XLOOKUP(G63,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC63" s="7">
+        <f>_xlfn.XLOOKUP(G63,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD63" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="64" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>165</v>
       </c>
@@ -7382,8 +9309,35 @@
         <f>_xlfn.XLOOKUP(P64,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.25</v>
       </c>
+      <c r="X64" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M64,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sumatera Utara</v>
+      </c>
+      <c r="Y64" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M64,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z64" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G64,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA64" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G64,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Overnight</v>
+      </c>
+      <c r="AB64" s="1">
+        <f>_xlfn.XLOOKUP(G64,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>1</v>
+      </c>
+      <c r="AC64" s="7">
+        <f>_xlfn.XLOOKUP(G64,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>25000</v>
+      </c>
+      <c r="AD64" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="65" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>166</v>
       </c>
@@ -7464,8 +9418,35 @@
         <f>_xlfn.XLOOKUP(P65,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.9</v>
       </c>
+      <c r="X65" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M65,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y65" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M65,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z65" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G65,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA65" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G65,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB65" s="1">
+        <f>_xlfn.XLOOKUP(G65,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC65" s="7">
+        <f>_xlfn.XLOOKUP(G65,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD65" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="66" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>168</v>
       </c>
@@ -7546,8 +9527,35 @@
         <f>_xlfn.XLOOKUP(P66,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.8</v>
       </c>
+      <c r="X66" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M66,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y66" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M66,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z66" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G66,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA66" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G66,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB66" s="1">
+        <f>_xlfn.XLOOKUP(G66,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC66" s="7">
+        <f>_xlfn.XLOOKUP(G66,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD66" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="67" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>169</v>
       </c>
@@ -7628,8 +9636,35 @@
         <f>_xlfn.XLOOKUP(P67,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.35</v>
       </c>
+      <c r="X67" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M67,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y67" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M67,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z67" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G67,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA67" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G67,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB67" s="1">
+        <f>_xlfn.XLOOKUP(G67,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC67" s="7">
+        <f>_xlfn.XLOOKUP(G67,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD67" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="68" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>171</v>
       </c>
@@ -7710,8 +9745,35 @@
         <f>_xlfn.XLOOKUP(P68,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.8</v>
       </c>
+      <c r="X68" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M68,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Banten</v>
+      </c>
+      <c r="Y68" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M68,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z68" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G68,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA68" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G68,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB68" s="1">
+        <f>_xlfn.XLOOKUP(G68,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC68" s="7">
+        <f>_xlfn.XLOOKUP(G68,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD68" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="69" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>172</v>
       </c>
@@ -7792,8 +9854,35 @@
         <f>_xlfn.XLOOKUP(P69,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.25</v>
       </c>
+      <c r="X69" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M69,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Tengah</v>
+      </c>
+      <c r="Y69" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M69,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z69" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G69,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA69" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G69,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB69" s="1">
+        <f>_xlfn.XLOOKUP(G69,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC69" s="7">
+        <f>_xlfn.XLOOKUP(G69,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD69" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="70" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>174</v>
       </c>
@@ -7874,8 +9963,35 @@
         <f>_xlfn.XLOOKUP(P70,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.9</v>
       </c>
+      <c r="X70" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M70,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y70" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M70,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z70" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G70,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA70" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G70,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB70" s="1">
+        <f>_xlfn.XLOOKUP(G70,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC70" s="7">
+        <f>_xlfn.XLOOKUP(G70,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD70" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="71" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>176</v>
       </c>
@@ -7956,8 +10072,35 @@
         <f>_xlfn.XLOOKUP(P71,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.2</v>
       </c>
+      <c r="X71" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M71,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Tengah</v>
+      </c>
+      <c r="Y71" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M71,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z71" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G71,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA71" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G71,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB71" s="1">
+        <f>_xlfn.XLOOKUP(G71,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC71" s="7">
+        <f>_xlfn.XLOOKUP(G71,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD71" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="72" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>178</v>
       </c>
@@ -8038,8 +10181,35 @@
         <f>_xlfn.XLOOKUP(P72,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.8</v>
       </c>
+      <c r="X72" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M72,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Tengah</v>
+      </c>
+      <c r="Y72" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M72,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z72" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G72,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA72" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G72,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB72" s="1">
+        <f>_xlfn.XLOOKUP(G72,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC72" s="7">
+        <f>_xlfn.XLOOKUP(G72,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD72" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="73" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>179</v>
       </c>
@@ -8120,8 +10290,35 @@
         <f>_xlfn.XLOOKUP(P73,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.1</v>
       </c>
+      <c r="X73" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M73,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Tengah</v>
+      </c>
+      <c r="Y73" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M73,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z73" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G73,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA73" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G73,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB73" s="1">
+        <f>_xlfn.XLOOKUP(G73,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC73" s="7">
+        <f>_xlfn.XLOOKUP(G73,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD73" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="74" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>180</v>
       </c>
@@ -8202,8 +10399,35 @@
         <f>_xlfn.XLOOKUP(P74,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.4</v>
       </c>
+      <c r="X74" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M74,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sumatera Utara</v>
+      </c>
+      <c r="Y74" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M74,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z74" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G74,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA74" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G74,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB74" s="1">
+        <f>_xlfn.XLOOKUP(G74,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC74" s="7">
+        <f>_xlfn.XLOOKUP(G74,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD74" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="75" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>182</v>
       </c>
@@ -8284,8 +10508,35 @@
         <f>_xlfn.XLOOKUP(P75,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>1.2</v>
       </c>
+      <c r="X75" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M75,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y75" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M75,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z75" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G75,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA75" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G75,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB75" s="1">
+        <f>_xlfn.XLOOKUP(G75,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC75" s="7">
+        <f>_xlfn.XLOOKUP(G75,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD75" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="76" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>184</v>
       </c>
@@ -8366,8 +10617,35 @@
         <f>_xlfn.XLOOKUP(P76,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.8</v>
       </c>
+      <c r="X76" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M76,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y76" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M76,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z76" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G76,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA76" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G76,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB76" s="1">
+        <f>_xlfn.XLOOKUP(G76,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC76" s="7">
+        <f>_xlfn.XLOOKUP(G76,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD76" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="77" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>186</v>
       </c>
@@ -8448,8 +10726,35 @@
         <f>_xlfn.XLOOKUP(P77,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.35</v>
       </c>
+      <c r="X77" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M77,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y77" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M77,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z77" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G77,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA77" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G77,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB77" s="1">
+        <f>_xlfn.XLOOKUP(G77,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC77" s="7">
+        <f>_xlfn.XLOOKUP(G77,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD77" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="78" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>187</v>
       </c>
@@ -8530,8 +10835,35 @@
         <f>_xlfn.XLOOKUP(P78,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>4.5</v>
       </c>
+      <c r="X78" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M78,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y78" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M78,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z78" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G78,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA78" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G78,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Overnight</v>
+      </c>
+      <c r="AB78" s="1">
+        <f>_xlfn.XLOOKUP(G78,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>1</v>
+      </c>
+      <c r="AC78" s="7">
+        <f>_xlfn.XLOOKUP(G78,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>25000</v>
+      </c>
+      <c r="AD78" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="79" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>188</v>
       </c>
@@ -8612,8 +10944,35 @@
         <f>_xlfn.XLOOKUP(P79,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>1.1</v>
       </c>
+      <c r="X79" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M79,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sumatera Utara</v>
+      </c>
+      <c r="Y79" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M79,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z79" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G79,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA79" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G79,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB79" s="1">
+        <f>_xlfn.XLOOKUP(G79,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC79" s="7">
+        <f>_xlfn.XLOOKUP(G79,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD79" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="80" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>190</v>
       </c>
@@ -8694,8 +11053,35 @@
         <f>_xlfn.XLOOKUP(P80,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>4.5</v>
       </c>
+      <c r="X80" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M80,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Bali</v>
+      </c>
+      <c r="Y80" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M80,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z80" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G80,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA80" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G80,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Overnight</v>
+      </c>
+      <c r="AB80" s="1">
+        <f>_xlfn.XLOOKUP(G80,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>1</v>
+      </c>
+      <c r="AC80" s="7">
+        <f>_xlfn.XLOOKUP(G80,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>25000</v>
+      </c>
+      <c r="AD80" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="81" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>192</v>
       </c>
@@ -8776,8 +11162,35 @@
         <f>_xlfn.XLOOKUP(P81,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.2</v>
       </c>
+      <c r="X81" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M81,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DI Yogyakarta</v>
+      </c>
+      <c r="Y81" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M81,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z81" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G81,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA81" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G81,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB81" s="1">
+        <f>_xlfn.XLOOKUP(G81,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC81" s="7">
+        <f>_xlfn.XLOOKUP(G81,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD81" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="82" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>193</v>
       </c>
@@ -8858,8 +11271,35 @@
         <f>_xlfn.XLOOKUP(P82,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.9</v>
       </c>
+      <c r="X82" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M82,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Tengah</v>
+      </c>
+      <c r="Y82" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M82,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z82" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G82,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA82" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G82,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB82" s="1">
+        <f>_xlfn.XLOOKUP(G82,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC82" s="7">
+        <f>_xlfn.XLOOKUP(G82,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD82" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="83" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>194</v>
       </c>
@@ -8940,8 +11380,35 @@
         <f>_xlfn.XLOOKUP(P83,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.3</v>
       </c>
+      <c r="X83" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M83,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Banten</v>
+      </c>
+      <c r="Y83" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M83,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z83" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G83,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA83" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G83,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB83" s="1">
+        <f>_xlfn.XLOOKUP(G83,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC83" s="7">
+        <f>_xlfn.XLOOKUP(G83,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD83" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="84" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>195</v>
       </c>
@@ -9022,8 +11489,35 @@
         <f>_xlfn.XLOOKUP(P84,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>4.5</v>
       </c>
+      <c r="X84" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M84,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Banten</v>
+      </c>
+      <c r="Y84" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M84,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z84" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G84,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA84" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G84,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Overnight</v>
+      </c>
+      <c r="AB84" s="1">
+        <f>_xlfn.XLOOKUP(G84,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>1</v>
+      </c>
+      <c r="AC84" s="7">
+        <f>_xlfn.XLOOKUP(G84,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>25000</v>
+      </c>
+      <c r="AD84" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="85" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>196</v>
       </c>
@@ -9104,8 +11598,35 @@
         <f>_xlfn.XLOOKUP(P85,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.3</v>
       </c>
+      <c r="X85" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M85,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sumatera Utara</v>
+      </c>
+      <c r="Y85" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M85,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z85" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G85,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA85" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G85,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB85" s="1">
+        <f>_xlfn.XLOOKUP(G85,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC85" s="7">
+        <f>_xlfn.XLOOKUP(G85,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD85" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="86" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>199</v>
       </c>
@@ -9186,8 +11707,35 @@
         <f>_xlfn.XLOOKUP(P86,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.12</v>
       </c>
+      <c r="X86" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M86,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y86" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M86,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z86" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G86,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA86" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G86,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB86" s="1">
+        <f>_xlfn.XLOOKUP(G86,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC86" s="7">
+        <f>_xlfn.XLOOKUP(G86,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD86" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="87" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>200</v>
       </c>
@@ -9268,8 +11816,35 @@
         <f>_xlfn.XLOOKUP(P87,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>1.1</v>
       </c>
+      <c r="X87" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M87,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Timur</v>
+      </c>
+      <c r="Y87" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M87,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z87" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G87,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA87" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G87,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Overnight</v>
+      </c>
+      <c r="AB87" s="1">
+        <f>_xlfn.XLOOKUP(G87,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>1</v>
+      </c>
+      <c r="AC87" s="7">
+        <f>_xlfn.XLOOKUP(G87,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>25000</v>
+      </c>
+      <c r="AD87" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="88" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>202</v>
       </c>
@@ -9350,8 +11925,35 @@
         <f>_xlfn.XLOOKUP(P88,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.4</v>
       </c>
+      <c r="X88" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M88,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sulawesi Selatan</v>
+      </c>
+      <c r="Y88" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M88,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z88" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G88,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA88" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G88,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB88" s="1">
+        <f>_xlfn.XLOOKUP(G88,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC88" s="7">
+        <f>_xlfn.XLOOKUP(G88,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD88" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="89" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>203</v>
       </c>
@@ -9432,8 +12034,35 @@
         <f>_xlfn.XLOOKUP(P89,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.9</v>
       </c>
+      <c r="X89" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M89,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sumatera Utara</v>
+      </c>
+      <c r="Y89" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M89,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z89" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G89,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA89" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G89,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB89" s="1">
+        <f>_xlfn.XLOOKUP(G89,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC89" s="7">
+        <f>_xlfn.XLOOKUP(G89,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD89" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="90" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>205</v>
       </c>
@@ -9514,8 +12143,35 @@
         <f>_xlfn.XLOOKUP(P90,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.8</v>
       </c>
+      <c r="X90" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M90,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DI Yogyakarta</v>
+      </c>
+      <c r="Y90" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M90,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z90" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G90,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA90" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G90,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB90" s="1">
+        <f>_xlfn.XLOOKUP(G90,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC90" s="7">
+        <f>_xlfn.XLOOKUP(G90,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD90" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="91" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>206</v>
       </c>
@@ -9596,8 +12252,35 @@
         <f>_xlfn.XLOOKUP(P91,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.9</v>
       </c>
+      <c r="X91" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M91,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Bali</v>
+      </c>
+      <c r="Y91" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M91,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z91" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G91,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA91" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G91,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB91" s="1">
+        <f>_xlfn.XLOOKUP(G91,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC91" s="7">
+        <f>_xlfn.XLOOKUP(G91,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD91" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="92" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>207</v>
       </c>
@@ -9678,8 +12361,35 @@
         <f>_xlfn.XLOOKUP(P92,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.1</v>
       </c>
+      <c r="X92" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M92,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sumatera Utara</v>
+      </c>
+      <c r="Y92" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M92,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z92" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G92,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA92" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G92,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Overnight</v>
+      </c>
+      <c r="AB92" s="1">
+        <f>_xlfn.XLOOKUP(G92,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>1</v>
+      </c>
+      <c r="AC92" s="7">
+        <f>_xlfn.XLOOKUP(G92,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>25000</v>
+      </c>
+      <c r="AD92" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="93" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>209</v>
       </c>
@@ -9760,8 +12470,35 @@
         <f>_xlfn.XLOOKUP(P93,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.8</v>
       </c>
+      <c r="X93" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M93,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sulawesi Selatan</v>
+      </c>
+      <c r="Y93" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M93,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z93" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G93,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA93" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G93,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB93" s="1">
+        <f>_xlfn.XLOOKUP(G93,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC93" s="7">
+        <f>_xlfn.XLOOKUP(G93,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD93" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="94" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>211</v>
       </c>
@@ -9842,8 +12579,35 @@
         <f>_xlfn.XLOOKUP(P94,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.8</v>
       </c>
+      <c r="X94" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M94,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Tengah</v>
+      </c>
+      <c r="Y94" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M94,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z94" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G94,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>JNE</v>
+      </c>
+      <c r="AA94" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G94,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB94" s="1">
+        <f>_xlfn.XLOOKUP(G94,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>3</v>
+      </c>
+      <c r="AC94" s="7">
+        <f>_xlfn.XLOOKUP(G94,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>12000</v>
+      </c>
+      <c r="AD94" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="95" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>213</v>
       </c>
@@ -9924,8 +12688,35 @@
         <f>_xlfn.XLOOKUP(P95,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.35</v>
       </c>
+      <c r="X95" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M95,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sulawesi Selatan</v>
+      </c>
+      <c r="Y95" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M95,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Silver</v>
+      </c>
+      <c r="Z95" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G95,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA95" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G95,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB95" s="1">
+        <f>_xlfn.XLOOKUP(G95,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC95" s="7">
+        <f>_xlfn.XLOOKUP(G95,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD95" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="96" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>214</v>
       </c>
@@ -10006,8 +12797,35 @@
         <f>_xlfn.XLOOKUP(P96,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>1.2</v>
       </c>
+      <c r="X96" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M96,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Bali</v>
+      </c>
+      <c r="Y96" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M96,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z96" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G96,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA96" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G96,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB96" s="1">
+        <f>_xlfn.XLOOKUP(G96,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC96" s="7">
+        <f>_xlfn.XLOOKUP(G96,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD96" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="97" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>215</v>
       </c>
@@ -10088,8 +12906,35 @@
         <f>_xlfn.XLOOKUP(P97,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>1.1</v>
       </c>
+      <c r="X97" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M97,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y97" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M97,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z97" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G97,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA97" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G97,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB97" s="1">
+        <f>_xlfn.XLOOKUP(G97,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC97" s="7">
+        <f>_xlfn.XLOOKUP(G97,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD97" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="98" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>217</v>
       </c>
@@ -10170,8 +13015,35 @@
         <f>_xlfn.XLOOKUP(P98,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.3</v>
       </c>
+      <c r="X98" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M98,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Sumatera Utara</v>
+      </c>
+      <c r="Y98" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M98,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z98" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G98,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA98" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G98,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Cargo</v>
+      </c>
+      <c r="AB98" s="1">
+        <f>_xlfn.XLOOKUP(G98,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>5</v>
+      </c>
+      <c r="AC98" s="7">
+        <f>_xlfn.XLOOKUP(G98,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>8000</v>
+      </c>
+      <c r="AD98" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="99" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>219</v>
       </c>
@@ -10252,8 +13124,35 @@
         <f>_xlfn.XLOOKUP(P99,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>4.5</v>
       </c>
+      <c r="X99" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M99,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Barat</v>
+      </c>
+      <c r="Y99" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M99,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>VIP</v>
+      </c>
+      <c r="Z99" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G99,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA99" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G99,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Regular</v>
+      </c>
+      <c r="AB99" s="1">
+        <f>_xlfn.XLOOKUP(G99,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>4</v>
+      </c>
+      <c r="AC99" s="7">
+        <f>_xlfn.XLOOKUP(G99,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>10000</v>
+      </c>
+      <c r="AD99" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="100" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>220</v>
       </c>
@@ -10334,8 +13233,35 @@
         <f>_xlfn.XLOOKUP(P100,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>3.2</v>
       </c>
+      <c r="X100" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M100,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="Y100" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M100,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Gold</v>
+      </c>
+      <c r="Z100" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G100,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>J&amp;T Express</v>
+      </c>
+      <c r="AA100" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G100,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB100" s="1">
+        <f>_xlfn.XLOOKUP(G100,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC100" s="7">
+        <f>_xlfn.XLOOKUP(G100,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>15000</v>
+      </c>
+      <c r="AD100" s="1" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
-    <row r="101" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>221</v>
       </c>
@@ -10415,6 +13341,33 @@
       <c r="W101" s="1" t="str">
         <f>_xlfn.XLOOKUP(P101,[2]Master_Product_Catalog!$A$2:$A$16,[2]Master_Product_Catalog!$G$2:$G$16,"Nothing")</f>
         <v>0.3</v>
+      </c>
+      <c r="X101" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M101,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$D$2:$D$11)</f>
+        <v>Jawa Tengah</v>
+      </c>
+      <c r="Y101" s="1" t="str">
+        <f>_xlfn.XLOOKUP(M101,[1]Master_Customer_Profile!$A$2:$A$11,[1]Master_Customer_Profile!$G$2:$G$11)</f>
+        <v>Platinum</v>
+      </c>
+      <c r="Z101" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G101,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$B$2:$B$7)</f>
+        <v>SiCepat</v>
+      </c>
+      <c r="AA101" s="1" t="str">
+        <f>_xlfn.XLOOKUP(G101,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$C$2:$C$7)</f>
+        <v>Express</v>
+      </c>
+      <c r="AB101" s="1">
+        <f>_xlfn.XLOOKUP(G101,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$D$2:$D$7)</f>
+        <v>2</v>
+      </c>
+      <c r="AC101" s="7">
+        <f>_xlfn.XLOOKUP(G101,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
+        <v>16000</v>
+      </c>
+      <c r="AD101" s="1" t="e">
+        <v>#N/A</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Exam Excel: advance INDEX MATC completed
</commit_message>
<xml_diff>
--- a/Exam/Excel/advanced_assessment_project/Raw_Transactions_2024_finish.xlsx
+++ b/Exam/Excel/advanced_assessment_project/Raw_Transactions_2024_finish.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\Project\Data-Analyst\Exam\Excel\advanced_assessment_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59A8E13B-F97A-4E0D-B2F6-BDDED7910EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AB02D64-0268-481D-92B3-6BDD6F6B67F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{56521A79-FDF7-45C8-BAA3-ABC64B3F8849}"/>
   </bookViews>
@@ -19,6 +19,7 @@
     <externalReference r:id="rId2"/>
     <externalReference r:id="rId3"/>
     <externalReference r:id="rId4"/>
+    <externalReference r:id="rId5"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,28 +36,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2027,6 +2006,105 @@
 </externalLink>
 </file>
 
+<file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Master_Commission_Rule"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="1">
+          <cell r="B1" t="str">
+            <v>VIP</v>
+          </cell>
+          <cell r="C1" t="str">
+            <v>Gold</v>
+          </cell>
+          <cell r="D1" t="str">
+            <v>Silver</v>
+          </cell>
+          <cell r="E1" t="str">
+            <v>Standard</v>
+          </cell>
+        </row>
+        <row r="2">
+          <cell r="A2" t="str">
+            <v>Electronics</v>
+          </cell>
+          <cell r="B2" t="str">
+            <v>0.05</v>
+          </cell>
+          <cell r="C2" t="str">
+            <v>0.04</v>
+          </cell>
+          <cell r="D2" t="str">
+            <v>0.03</v>
+          </cell>
+          <cell r="E2" t="str">
+            <v>0.02</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="A3" t="str">
+            <v>Fashion</v>
+          </cell>
+          <cell r="B3" t="str">
+            <v>0.08</v>
+          </cell>
+          <cell r="C3" t="str">
+            <v>0.07</v>
+          </cell>
+          <cell r="D3" t="str">
+            <v>0.05</v>
+          </cell>
+          <cell r="E3" t="str">
+            <v>0.04</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="A4" t="str">
+            <v>Home &amp; Living</v>
+          </cell>
+          <cell r="B4" t="str">
+            <v>0.06</v>
+          </cell>
+          <cell r="C4" t="str">
+            <v>0.05</v>
+          </cell>
+          <cell r="D4" t="str">
+            <v>0.04</v>
+          </cell>
+          <cell r="E4" t="str">
+            <v>0.03</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="A5" t="str">
+            <v>Beauty &amp; Health</v>
+          </cell>
+          <cell r="B5" t="str">
+            <v>0.1</v>
+          </cell>
+          <cell r="C5" t="str">
+            <v>0.08</v>
+          </cell>
+          <cell r="D5" t="str">
+            <v>0.06</v>
+          </cell>
+          <cell r="E5" t="str">
+            <v>0.05</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2344,7 +2422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6A4B63D-0D46-44D9-8B15-778A85DACDCF}">
-  <dimension ref="A1:AD101"/>
+  <dimension ref="A1:AG101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
@@ -2377,7 +2455,7 @@
     <col min="30" max="30" width="22.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -2469,7 +2547,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -2574,12 +2652,12 @@
         <f>_xlfn.XLOOKUP(G2,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD2" s="1" t="e" cm="1">
-        <f t="array" ref="AD2:AD101">INDEX(MATCH(S2,S2:S101,0),MATCH(Y2:Y101,0))</f>
-        <v>#N/A</v>
+      <c r="AD2" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S2,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y2,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>20</v>
       </c>
@@ -2684,11 +2762,20 @@
         <f>_xlfn.XLOOKUP(G3,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD3" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD3" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S3,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y3,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
+      </c>
+      <c r="AF3">
+        <f>MATCH(S2,[4]Master_Commission_Rule!$A$2:$A$5,0)</f>
+        <v>1</v>
+      </c>
+      <c r="AG3">
+        <f>MATCH(Y4,[4]Master_Commission_Rule!$B$1:$E$1,0)</f>
+        <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>28</v>
       </c>
@@ -2793,11 +2880,12 @@
         <f>_xlfn.XLOOKUP(G4,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD4" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD4" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S4,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y4,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.08</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
@@ -2902,11 +2990,12 @@
         <f>_xlfn.XLOOKUP(G5,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD5" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD5" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S5,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y5,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.07</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>40</v>
       </c>
@@ -3011,11 +3100,12 @@
         <f>_xlfn.XLOOKUP(G6,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>25000</v>
       </c>
-      <c r="AD6" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD6" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S6,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y6,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.08</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>44</v>
       </c>
@@ -3120,11 +3210,12 @@
         <f>_xlfn.XLOOKUP(G7,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD7" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD7" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S7,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y7,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>49</v>
       </c>
@@ -3229,11 +3320,12 @@
         <f>_xlfn.XLOOKUP(G8,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>25000</v>
       </c>
-      <c r="AD8" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD8" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S8,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y8,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>51</v>
       </c>
@@ -3338,11 +3430,12 @@
         <f>_xlfn.XLOOKUP(G9,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD9" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD9" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S9,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y9,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>55</v>
       </c>
@@ -3447,11 +3540,12 @@
         <f>_xlfn.XLOOKUP(G10,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD10" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD10" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S10,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y10,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.03</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>58</v>
       </c>
@@ -3556,11 +3650,12 @@
         <f>_xlfn.XLOOKUP(G11,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD11" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD11" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S11,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y11,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>60</v>
       </c>
@@ -3665,11 +3760,12 @@
         <f>_xlfn.XLOOKUP(G12,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD12" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD12" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S12,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y12,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>63</v>
       </c>
@@ -3774,11 +3870,12 @@
         <f>_xlfn.XLOOKUP(G13,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD13" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD13" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S13,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y13,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>66</v>
       </c>
@@ -3883,11 +3980,12 @@
         <f>_xlfn.XLOOKUP(G14,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>8000</v>
       </c>
-      <c r="AD14" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD14" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S14,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y14,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>68</v>
       </c>
@@ -3992,11 +4090,12 @@
         <f>_xlfn.XLOOKUP(G15,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD15" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD15" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S15,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y15,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.03</v>
       </c>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>71</v>
       </c>
@@ -4101,8 +4200,9 @@
         <f>_xlfn.XLOOKUP(G16,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>8000</v>
       </c>
-      <c r="AD16" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD16" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S16,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y16,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
     <row r="17" spans="1:30" x14ac:dyDescent="0.25">
@@ -4210,8 +4310,9 @@
         <f>_xlfn.XLOOKUP(G17,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD17" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD17" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S17,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y17,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.08</v>
       </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.25">
@@ -4319,8 +4420,9 @@
         <f>_xlfn.XLOOKUP(G18,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD18" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD18" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S18,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y18,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
     <row r="19" spans="1:30" x14ac:dyDescent="0.25">
@@ -4428,8 +4530,9 @@
         <f>_xlfn.XLOOKUP(G19,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD19" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD19" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S19,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y19,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.03</v>
       </c>
     </row>
     <row r="20" spans="1:30" x14ac:dyDescent="0.25">
@@ -4537,8 +4640,9 @@
         <f>_xlfn.XLOOKUP(G20,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD20" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD20" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S20,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y20,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="21" spans="1:30" x14ac:dyDescent="0.25">
@@ -4646,8 +4750,9 @@
         <f>_xlfn.XLOOKUP(G21,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>8000</v>
       </c>
-      <c r="AD21" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD21" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S21,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y21,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
     <row r="22" spans="1:30" x14ac:dyDescent="0.25">
@@ -4756,6 +4861,7 @@
         <v>15000</v>
       </c>
       <c r="AD22" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S22,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y22,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -4864,8 +4970,9 @@
         <f>_xlfn.XLOOKUP(G23,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD23" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD23" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S23,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y23,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="24" spans="1:30" x14ac:dyDescent="0.25">
@@ -4973,8 +5080,9 @@
         <f>_xlfn.XLOOKUP(G24,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD24" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD24" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S24,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y24,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
     <row r="25" spans="1:30" x14ac:dyDescent="0.25">
@@ -5083,6 +5191,7 @@
         <v>12000</v>
       </c>
       <c r="AD25" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S25,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y25,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -5191,8 +5300,9 @@
         <f>_xlfn.XLOOKUP(G26,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD26" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD26" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S26,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y26,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="27" spans="1:30" x14ac:dyDescent="0.25">
@@ -5300,8 +5410,9 @@
         <f>_xlfn.XLOOKUP(G27,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD27" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD27" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S27,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y27,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.07</v>
       </c>
     </row>
     <row r="28" spans="1:30" x14ac:dyDescent="0.25">
@@ -5409,8 +5520,9 @@
         <f>_xlfn.XLOOKUP(G28,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD28" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD28" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S28,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y28,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="29" spans="1:30" x14ac:dyDescent="0.25">
@@ -5518,8 +5630,9 @@
         <f>_xlfn.XLOOKUP(G29,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD29" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD29" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S29,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y29,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="30" spans="1:30" x14ac:dyDescent="0.25">
@@ -5627,8 +5740,9 @@
         <f>_xlfn.XLOOKUP(G30,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD30" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD30" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S30,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y30,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="31" spans="1:30" x14ac:dyDescent="0.25">
@@ -5736,8 +5850,9 @@
         <f>_xlfn.XLOOKUP(G31,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>8000</v>
       </c>
-      <c r="AD31" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD31" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S31,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y31,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="32" spans="1:30" x14ac:dyDescent="0.25">
@@ -5845,8 +5960,9 @@
         <f>_xlfn.XLOOKUP(G32,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD32" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD32" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S32,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y32,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.08</v>
       </c>
     </row>
     <row r="33" spans="1:30" x14ac:dyDescent="0.25">
@@ -5954,8 +6070,9 @@
         <f>_xlfn.XLOOKUP(G33,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>8000</v>
       </c>
-      <c r="AD33" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD33" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S33,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y33,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.03</v>
       </c>
     </row>
     <row r="34" spans="1:30" x14ac:dyDescent="0.25">
@@ -6063,8 +6180,9 @@
         <f>_xlfn.XLOOKUP(G34,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD34" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD34" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S34,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y34,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="35" spans="1:30" x14ac:dyDescent="0.25">
@@ -6172,8 +6290,9 @@
         <f>_xlfn.XLOOKUP(G35,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD35" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD35" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S35,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y35,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.08</v>
       </c>
     </row>
     <row r="36" spans="1:30" x14ac:dyDescent="0.25">
@@ -6281,8 +6400,9 @@
         <f>_xlfn.XLOOKUP(G36,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD36" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD36" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S36,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y36,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.07</v>
       </c>
     </row>
     <row r="37" spans="1:30" x14ac:dyDescent="0.25">
@@ -6391,6 +6511,7 @@
         <v>25000</v>
       </c>
       <c r="AD37" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S37,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y37,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -6499,8 +6620,9 @@
         <f>_xlfn.XLOOKUP(G38,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD38" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD38" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S38,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y38,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.07</v>
       </c>
     </row>
     <row r="39" spans="1:30" x14ac:dyDescent="0.25">
@@ -6608,8 +6730,9 @@
         <f>_xlfn.XLOOKUP(G39,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>8000</v>
       </c>
-      <c r="AD39" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD39" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S39,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y39,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="40" spans="1:30" x14ac:dyDescent="0.25">
@@ -6717,8 +6840,9 @@
         <f>_xlfn.XLOOKUP(G40,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>25000</v>
       </c>
-      <c r="AD40" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD40" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S40,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y40,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="41" spans="1:30" x14ac:dyDescent="0.25">
@@ -6826,8 +6950,9 @@
         <f>_xlfn.XLOOKUP(G41,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD41" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD41" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S41,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y41,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.08</v>
       </c>
     </row>
     <row r="42" spans="1:30" x14ac:dyDescent="0.25">
@@ -6935,8 +7060,9 @@
         <f>_xlfn.XLOOKUP(G42,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>8000</v>
       </c>
-      <c r="AD42" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD42" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S42,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y42,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="43" spans="1:30" x14ac:dyDescent="0.25">
@@ -7045,6 +7171,7 @@
         <v>12000</v>
       </c>
       <c r="AD43" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S43,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y43,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -7153,8 +7280,9 @@
         <f>_xlfn.XLOOKUP(G44,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD44" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD44" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S44,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y44,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="45" spans="1:30" x14ac:dyDescent="0.25">
@@ -7262,8 +7390,9 @@
         <f>_xlfn.XLOOKUP(G45,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD45" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD45" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S45,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y45,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="46" spans="1:30" x14ac:dyDescent="0.25">
@@ -7371,8 +7500,9 @@
         <f>_xlfn.XLOOKUP(G46,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD46" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD46" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S46,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y46,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="47" spans="1:30" x14ac:dyDescent="0.25">
@@ -7480,8 +7610,9 @@
         <f>_xlfn.XLOOKUP(G47,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD47" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD47" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S47,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y47,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="48" spans="1:30" x14ac:dyDescent="0.25">
@@ -7590,6 +7721,7 @@
         <v>10000</v>
       </c>
       <c r="AD48" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S48,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y48,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -7698,8 +7830,9 @@
         <f>_xlfn.XLOOKUP(G49,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD49" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD49" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S49,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y49,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="50" spans="1:30" x14ac:dyDescent="0.25">
@@ -7807,8 +7940,9 @@
         <f>_xlfn.XLOOKUP(G50,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD50" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD50" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S50,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y50,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.08</v>
       </c>
     </row>
     <row r="51" spans="1:30" x14ac:dyDescent="0.25">
@@ -7916,8 +8050,9 @@
         <f>_xlfn.XLOOKUP(G51,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD51" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD51" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S51,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y51,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="52" spans="1:30" x14ac:dyDescent="0.25">
@@ -8025,8 +8160,9 @@
         <f>_xlfn.XLOOKUP(G52,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD52" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD52" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S52,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y52,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.03</v>
       </c>
     </row>
     <row r="53" spans="1:30" x14ac:dyDescent="0.25">
@@ -8134,8 +8270,9 @@
         <f>_xlfn.XLOOKUP(G53,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD53" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD53" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S53,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y53,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
     <row r="54" spans="1:30" x14ac:dyDescent="0.25">
@@ -8243,8 +8380,9 @@
         <f>_xlfn.XLOOKUP(G54,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD54" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD54" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S54,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y54,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
     <row r="55" spans="1:30" x14ac:dyDescent="0.25">
@@ -8353,6 +8491,7 @@
         <v>15000</v>
       </c>
       <c r="AD55" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S55,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y55,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -8461,8 +8600,9 @@
         <f>_xlfn.XLOOKUP(G56,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD56" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD56" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S56,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y56,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="57" spans="1:30" x14ac:dyDescent="0.25">
@@ -8571,6 +8711,7 @@
         <v>8000</v>
       </c>
       <c r="AD57" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S57,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y57,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -8679,8 +8820,9 @@
         <f>_xlfn.XLOOKUP(G58,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD58" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD58" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S58,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y58,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.1</v>
       </c>
     </row>
     <row r="59" spans="1:30" x14ac:dyDescent="0.25">
@@ -8788,8 +8930,9 @@
         <f>_xlfn.XLOOKUP(G59,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD59" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD59" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S59,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y59,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="60" spans="1:30" x14ac:dyDescent="0.25">
@@ -8897,8 +9040,9 @@
         <f>_xlfn.XLOOKUP(G60,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD60" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD60" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S60,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y60,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="61" spans="1:30" x14ac:dyDescent="0.25">
@@ -9006,8 +9150,9 @@
         <f>_xlfn.XLOOKUP(G61,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD61" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD61" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S61,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y61,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.1</v>
       </c>
     </row>
     <row r="62" spans="1:30" x14ac:dyDescent="0.25">
@@ -9116,6 +9261,7 @@
         <v>8000</v>
       </c>
       <c r="AD62" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S62,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y62,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -9224,8 +9370,9 @@
         <f>_xlfn.XLOOKUP(G63,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD63" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD63" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S63,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y63,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="64" spans="1:30" x14ac:dyDescent="0.25">
@@ -9333,8 +9480,9 @@
         <f>_xlfn.XLOOKUP(G64,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>25000</v>
       </c>
-      <c r="AD64" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD64" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S64,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y64,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="65" spans="1:30" x14ac:dyDescent="0.25">
@@ -9442,8 +9590,9 @@
         <f>_xlfn.XLOOKUP(G65,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD65" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD65" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S65,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y65,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="66" spans="1:30" x14ac:dyDescent="0.25">
@@ -9551,8 +9700,9 @@
         <f>_xlfn.XLOOKUP(G66,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD66" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD66" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S66,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y66,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="67" spans="1:30" x14ac:dyDescent="0.25">
@@ -9660,8 +9810,9 @@
         <f>_xlfn.XLOOKUP(G67,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD67" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD67" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S67,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y67,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="68" spans="1:30" x14ac:dyDescent="0.25">
@@ -9769,8 +9920,9 @@
         <f>_xlfn.XLOOKUP(G68,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD68" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD68" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S68,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y68,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="69" spans="1:30" x14ac:dyDescent="0.25">
@@ -9879,6 +10031,7 @@
         <v>15000</v>
       </c>
       <c r="AD69" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S69,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y69,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -9987,8 +10140,9 @@
         <f>_xlfn.XLOOKUP(G70,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD70" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD70" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S70,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y70,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="71" spans="1:30" x14ac:dyDescent="0.25">
@@ -10097,6 +10251,7 @@
         <v>12000</v>
       </c>
       <c r="AD71" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S71,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y71,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -10206,6 +10361,7 @@
         <v>16000</v>
       </c>
       <c r="AD72" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S72,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y72,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -10315,6 +10471,7 @@
         <v>16000</v>
       </c>
       <c r="AD73" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S73,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y73,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -10423,8 +10580,9 @@
         <f>_xlfn.XLOOKUP(G74,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD74" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD74" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S74,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y74,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="75" spans="1:30" x14ac:dyDescent="0.25">
@@ -10532,8 +10690,9 @@
         <f>_xlfn.XLOOKUP(G75,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>8000</v>
       </c>
-      <c r="AD75" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD75" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S75,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y75,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="76" spans="1:30" x14ac:dyDescent="0.25">
@@ -10641,8 +10800,9 @@
         <f>_xlfn.XLOOKUP(G76,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>8000</v>
       </c>
-      <c r="AD76" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD76" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S76,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y76,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="77" spans="1:30" x14ac:dyDescent="0.25">
@@ -10750,8 +10910,9 @@
         <f>_xlfn.XLOOKUP(G77,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD77" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD77" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S77,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y77,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="78" spans="1:30" x14ac:dyDescent="0.25">
@@ -10859,8 +11020,9 @@
         <f>_xlfn.XLOOKUP(G78,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>25000</v>
       </c>
-      <c r="AD78" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD78" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S78,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y78,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="79" spans="1:30" x14ac:dyDescent="0.25">
@@ -10968,8 +11130,9 @@
         <f>_xlfn.XLOOKUP(G79,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD79" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD79" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S79,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y79,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.07</v>
       </c>
     </row>
     <row r="80" spans="1:30" x14ac:dyDescent="0.25">
@@ -11077,8 +11240,9 @@
         <f>_xlfn.XLOOKUP(G80,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>25000</v>
       </c>
-      <c r="AD80" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD80" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S80,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y80,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
     <row r="81" spans="1:30" x14ac:dyDescent="0.25">
@@ -11187,6 +11351,7 @@
         <v>8000</v>
       </c>
       <c r="AD81" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S81,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y81,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -11296,6 +11461,7 @@
         <v>15000</v>
       </c>
       <c r="AD82" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S82,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y82,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -11404,8 +11570,9 @@
         <f>_xlfn.XLOOKUP(G83,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD83" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD83" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S83,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y83,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.03</v>
       </c>
     </row>
     <row r="84" spans="1:30" x14ac:dyDescent="0.25">
@@ -11513,8 +11680,9 @@
         <f>_xlfn.XLOOKUP(G84,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>25000</v>
       </c>
-      <c r="AD84" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD84" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S84,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y84,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="85" spans="1:30" x14ac:dyDescent="0.25">
@@ -11622,8 +11790,9 @@
         <f>_xlfn.XLOOKUP(G85,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD85" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD85" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S85,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y85,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="86" spans="1:30" x14ac:dyDescent="0.25">
@@ -11731,8 +11900,9 @@
         <f>_xlfn.XLOOKUP(G86,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD86" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD86" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S86,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y86,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
     <row r="87" spans="1:30" x14ac:dyDescent="0.25">
@@ -11840,8 +12010,9 @@
         <f>_xlfn.XLOOKUP(G87,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>25000</v>
       </c>
-      <c r="AD87" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD87" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S87,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y87,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="88" spans="1:30" x14ac:dyDescent="0.25">
@@ -11949,8 +12120,9 @@
         <f>_xlfn.XLOOKUP(G88,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD88" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD88" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S88,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y88,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.03</v>
       </c>
     </row>
     <row r="89" spans="1:30" x14ac:dyDescent="0.25">
@@ -12058,8 +12230,9 @@
         <f>_xlfn.XLOOKUP(G89,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD89" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD89" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S89,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y89,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.07</v>
       </c>
     </row>
     <row r="90" spans="1:30" x14ac:dyDescent="0.25">
@@ -12168,6 +12341,7 @@
         <v>15000</v>
       </c>
       <c r="AD90" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S90,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y90,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -12276,8 +12450,9 @@
         <f>_xlfn.XLOOKUP(G91,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>12000</v>
       </c>
-      <c r="AD91" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD91" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S91,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y91,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.08</v>
       </c>
     </row>
     <row r="92" spans="1:30" x14ac:dyDescent="0.25">
@@ -12385,8 +12560,9 @@
         <f>_xlfn.XLOOKUP(G92,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>25000</v>
       </c>
-      <c r="AD92" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD92" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S92,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y92,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.08</v>
       </c>
     </row>
     <row r="93" spans="1:30" x14ac:dyDescent="0.25">
@@ -12494,8 +12670,9 @@
         <f>_xlfn.XLOOKUP(G93,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD93" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD93" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S93,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y93,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.03</v>
       </c>
     </row>
     <row r="94" spans="1:30" x14ac:dyDescent="0.25">
@@ -12604,6 +12781,7 @@
         <v>12000</v>
       </c>
       <c r="AD94" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S94,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y94,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -12712,8 +12890,9 @@
         <f>_xlfn.XLOOKUP(G95,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>16000</v>
       </c>
-      <c r="AD95" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD95" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S95,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y95,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="96" spans="1:30" x14ac:dyDescent="0.25">
@@ -12821,8 +13000,9 @@
         <f>_xlfn.XLOOKUP(G96,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>8000</v>
       </c>
-      <c r="AD96" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD96" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S96,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y96,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="97" spans="1:30" x14ac:dyDescent="0.25">
@@ -12930,8 +13110,9 @@
         <f>_xlfn.XLOOKUP(G97,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD97" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD97" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S97,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y97,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.07</v>
       </c>
     </row>
     <row r="98" spans="1:30" x14ac:dyDescent="0.25">
@@ -13039,8 +13220,9 @@
         <f>_xlfn.XLOOKUP(G98,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>8000</v>
       </c>
-      <c r="AD98" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD98" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S98,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y98,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.04</v>
       </c>
     </row>
     <row r="99" spans="1:30" x14ac:dyDescent="0.25">
@@ -13148,8 +13330,9 @@
         <f>_xlfn.XLOOKUP(G99,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>10000</v>
       </c>
-      <c r="AD99" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD99" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S99,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y99,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.06</v>
       </c>
     </row>
     <row r="100" spans="1:30" x14ac:dyDescent="0.25">
@@ -13257,8 +13440,9 @@
         <f>_xlfn.XLOOKUP(G100,[3]Master_SLA_Shipping!$A$2:$A$7,[3]Master_SLA_Shipping!$E$2:$E$7)</f>
         <v>15000</v>
       </c>
-      <c r="AD100" s="1" t="e">
-        <v>#N/A</v>
+      <c r="AD100" s="1" t="str">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S100,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y100,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="101" spans="1:30" x14ac:dyDescent="0.25">
@@ -13367,6 +13551,7 @@
         <v>16000</v>
       </c>
       <c r="AD101" s="1" t="e">
+        <f>INDEX([4]Master_Commission_Rule!$B$2:$E$5,MATCH(S101,[4]Master_Commission_Rule!$A$2:$A$5,0),MATCH(Y101,[4]Master_Commission_Rule!$B$1:$E$1,0))</f>
         <v>#N/A</v>
       </c>
     </row>

</xml_diff>